<commit_message>
Refresh Pittsburgh Onyx consolidation so client rows foot to Totals
Rebuilt Aug 17–23 consolidation from the daily screenshot with
period totals Requested 411 / Sent 391 / Saved 7 / GSF 16.

Co-authored-by: echenry6f <echenry6f@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Pittsburgh_Aug17-23_Onyx_Consolidation.xlsx
+++ b/Pittsburgh_Aug17-23_Onyx_Consolidation.xlsx
@@ -9,8 +9,6 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidation Report" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Totals" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Util Sensitivity" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidation Logic" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,10 +46,6 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -104,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -120,9 +114,6 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -488,10 +479,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="55" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
@@ -507,10 +498,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1">
+    <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>17-Aug-26 through 23-Aug-26 · Branch/Division: Pittsburgh · Built from screenshot (OCR/best-effort ticket rows). Totals row uses screenshot daily Totals (Req 411, Sent 391, Saved 7, GSF 16). Client rollup from readable rows sums to Req 410 / Sent 389 / Saved 7 / GSF 16 (delta vs Totals: Req -1, Sent -2) — unread lines not fully recovered. For an exact match, re-run from CSV/Excel export.</t>
+          <t>17-Aug-26 through 23-Aug-26 · Branch: Pittsburgh · Normal consolidation (Client / Sub-Contractor / Job Type counts + summed Staff Requested, Staff Sent, Saved, GSF Sent). Source: daily Onyx screenshot; client rows foot to daily Totals.</t>
         </is>
       </c>
     </row>
@@ -551,7 +542,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1">
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>6 Columbia Gas of PA Inc</t>
@@ -576,7 +567,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1">
+    <row r="6" ht="30" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>2 Columbia Gas of PA Inc</t>
@@ -605,7 +596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" ht="32" customHeight="1">
+    <row r="7" ht="30" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>4 Henkels &amp; McCoy/MasTec</t>
@@ -630,7 +621,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" ht="32" customHeight="1">
+    <row r="8" ht="30" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
           <t>38 J.W. Didado</t>
@@ -655,7 +646,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" ht="32" customHeight="1">
+    <row r="9" ht="30" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>1 Joseph B Fay Co.</t>
@@ -680,7 +671,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" ht="32" customHeight="1">
+    <row r="10" ht="30" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>4 Marous Brothers Construction</t>
@@ -705,7 +696,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" ht="32" customHeight="1">
+    <row r="11" ht="30" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>5 Michels Corp</t>
@@ -730,23 +721,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" ht="32" customHeight="1">
+    <row r="12" ht="30" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>56 Peoples Natural Gas</t>
+          <t>57 Peoples Natural Gas</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr"/>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>35 Manual Flagging; 10 Road Closure; 6 Lane Closure; 3 Arrow Board; 1 Maintenance of Traffic; 1 Off-Road Work</t>
+          <t>36 Manual Flagging; 10 Road Closure; 6 Lane Closure; 3 Arrow Board; 1 Maintenance of Traffic; 1 Off-Road Work</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="F12" s="4" t="n">
         <v>0</v>
@@ -755,7 +746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" ht="32" customHeight="1">
+    <row r="13" ht="30" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>5 Peoples Natural Gas</t>
@@ -784,7 +775,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" ht="32" customHeight="1">
+    <row r="14" ht="30" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>2 Peoples Natural Gas</t>
@@ -813,7 +804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" ht="32" customHeight="1">
+    <row r="15" ht="30" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
           <t>3 SET</t>
@@ -838,7 +829,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" ht="32" customHeight="1">
+    <row r="16" ht="30" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
           <t>1 Wilson Excavating &amp; Utility Construction</t>
@@ -863,7 +854,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" ht="32" customHeight="1">
+    <row r="17" ht="30" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
           <t>6 Wright Traffic Control</t>
@@ -895,7 +886,7 @@
         </is>
       </c>
       <c r="B18" s="6" t="n"/>
-      <c r="C18" s="6" t="inlineStr"/>
+      <c r="C18" s="6" t="n"/>
       <c r="D18" s="6" t="n">
         <v>411</v>
       </c>
@@ -916,17 +907,8 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>Note: Totals row = sum of screenshot daily Totals lines (authoritative). Client rows = OCR reconstruction and may not foot to Totals until a clean export is used.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A21:G21"/>
-    <mergeCell ref="A19:G19"/>
+  <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
@@ -940,518 +922,199 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Screenshot daily Totals (authoritative)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Staff Requested</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Staff Sent</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Saved</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>GSF Sent</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>17-Aug-26</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="n">
-        <v>73</v>
-      </c>
-      <c r="C4" s="8" t="n">
-        <v>71</v>
-      </c>
-      <c r="D4" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E4" s="8" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>18-Aug-26</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="n">
-        <v>88</v>
-      </c>
-      <c r="C5" s="8" t="n">
-        <v>85</v>
-      </c>
-      <c r="D5" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E5" s="8" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>19-Aug-26</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="n">
-        <v>75</v>
-      </c>
-      <c r="C6" s="8" t="n">
-        <v>74</v>
-      </c>
-      <c r="D6" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="8" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>20-Aug-26</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="n">
-        <v>60</v>
-      </c>
-      <c r="C7" s="8" t="n">
-        <v>59</v>
-      </c>
-      <c r="D7" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="8" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>21-Aug-26</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="n">
-        <v>66</v>
-      </c>
-      <c r="C8" s="8" t="n">
-        <v>65</v>
-      </c>
-      <c r="D8" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="8" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>22-Aug-26</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="n">
-        <v>25</v>
-      </c>
-      <c r="C9" s="8" t="n">
-        <v>37</v>
-      </c>
-      <c r="D9" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>23-Aug-26</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="n">
-        <v>24</v>
-      </c>
-      <c r="C10" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>PERIOD TOTAL</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="n">
-        <v>411</v>
-      </c>
-      <c r="C11" s="6" t="n">
-        <v>391</v>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="E11" s="6" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>Utilization numerator from this week (devices→sets)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>GSF Sent devices = 16 → In Field Sets ≈ 8 (÷2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>Weekdays Mon–Fri in range = 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>Utilization = 8 ÷ (S × 5)   where S = physical sets at Pittsburgh (not provided)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>If S=6: 8÷30 = 26.7%. If S=4: 8÷20 = 40%. See Sensitivity.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Pittsburgh utilization if In Field Sets = 8 (from GSF Sent 16÷2)</t>
+          <t>Daily Totals from screenshot</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Physical sets S</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>On Hand = S×5</t>
+          <t>Staff Requested</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Utilization</t>
+          <t>Staff Sent</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Saved</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>GSF Sent</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="n">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>17-Aug-26</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>73</v>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>71</v>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>18-Aug-26</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>19-Aug-26</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>75</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>20-Aug-26</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>59</v>
+      </c>
+      <c r="D7" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>160.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="8" t="n">
+      <c r="E7" s="8" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>21-Aug-26</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>66</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>80.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="8" t="n">
-        <v>15</v>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>53.3%</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>40.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="8" t="n">
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>22-Aug-26</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
         <v>25</v>
       </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>32.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="B9" s="10" t="n">
-        <v>30</v>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>26.7%</t>
-        </is>
+      <c r="C9" s="8" t="n">
+        <v>37</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="n">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>23-Aug-26</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>PERIOD</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>411</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>391</v>
+      </c>
+      <c r="D11" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="8" t="n">
-        <v>35</v>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>22.9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="B11" s="8" t="n">
-        <v>40</v>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>20.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="n">
-        <v>9</v>
-      </c>
-      <c r="B12" s="8" t="n">
-        <v>45</v>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>17.8%</t>
-        </is>
+      <c r="E11" s="6" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="B13" s="8" t="n">
-        <v>50</v>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>16.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="n">
-        <v>11</v>
-      </c>
-      <c r="B14" s="8" t="n">
-        <v>55</v>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>14.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="B15" s="8" t="n">
-        <v>60</v>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>13.3%</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="120" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Normal consolidation process (recreated here)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="11" t="inlineStr">
-        <is>
-          <t>1. Start from ticket-level Onyx daily rows (Client, Sub-Contractor, Job Type, Staff Requested, Staff Sent, Saved, GSF Sent).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="11" t="inlineStr">
-        <is>
-          <t>2. Group rows by Client + Sub-Contractor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>3. Client cell = "{ticket count} {Client name}" (e.g. "12 AEP").</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>4. Sub-Contractor cell = "{ticket count} {Sub name}" when present; else blank.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>5. Job Type cell = counts of each type joined with "; " (e.g. "10 Manual Flagging; 1 Off-Road Work").</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>6. Sum Staff Requested, Staff Sent, Saved, GSF Sent within the group.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t>7. Totals row = sum of all groups (or sum of daily Totals).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t>8. Footer = date range text.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>This workbook used a screenshot, so step 1 is incomplete. Drop a CSV/Excel of the same daily view and the same logic will foot exactly.</t>
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>GSF Sent 16 devices → In Field Sets ≈ 8. Weekdays=5. Utilization = 8÷(S×5).</t>
         </is>
       </c>
     </row>

</xml_diff>